<commit_message>
refactor(config)!: inline additional costs with integer resource IDs
</commit_message>
<xml_diff>
--- a/config/tables/gas.ability.xlsx
+++ b/config/tables/gas.ability.xlsx
@@ -1238,7 +1238,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>additional_cost_ids</t>
+          <t>additional_costs</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>(list#sep=;),(int#ref=gas.TbAbilityAdditionalCost)</t>
+          <t>(list#sep=;),gas.AbilityAdditionalCost</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Additional cost IDs in payment order. Blank means none.</t>
+          <t>Ordered integer resource ID,amount pairs separated by semicolons. Blank means none.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>10021</t>
+          <t>5001,1</t>
         </is>
       </c>
       <c r="G6" s="9" t="n"/>

</xml_diff>